<commit_message>
chore: update 产品库存及周转统计 workbook
</commit_message>
<xml_diff>
--- a/dist/产品库存及周转统计.xlsx
+++ b/dist/产品库存及周转统计.xlsx
@@ -4,20 +4,20 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="16160"/>
+    <workbookView windowHeight="15240"/>
   </bookViews>
   <sheets>
     <sheet name="产品库存" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">产品库存!$A$1:$AH$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">产品库存!$A$1:$AH$60</definedName>
   </definedNames>
   <calcPr calcId="144525" concurrentCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="276">
   <si>
     <t>名称</t>
   </si>
@@ -835,6 +835,30 @@
   </si>
   <si>
     <t>X005166XCN</t>
+  </si>
+  <si>
+    <t>【小】灰色B款(2p)</t>
+  </si>
+  <si>
+    <t>B0GWWS56G5</t>
+  </si>
+  <si>
+    <t>WallHangingBagSmallGray_2P_B</t>
+  </si>
+  <si>
+    <t>X0052N791J</t>
+  </si>
+  <si>
+    <t>【小】白色B款(2p)</t>
+  </si>
+  <si>
+    <t>B0GWWP5MT7</t>
+  </si>
+  <si>
+    <t>WallHangingBagSmallWhite_2P_B</t>
+  </si>
+  <si>
+    <t>X0052N76DZ</t>
   </si>
 </sst>
 </file>
@@ -2165,7 +2189,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="27">
-        <f t="shared" ref="E2:E60" si="0">C2+D2</f>
+        <f t="shared" ref="E2:E62" si="0">C2+D2</f>
         <v>0</v>
       </c>
       <c r="F2" s="28">
@@ -2182,11 +2206,11 @@
         <v>22.55</v>
       </c>
       <c r="J2" s="26">
-        <f t="shared" ref="J2:J60" si="2">(C2)/I2</f>
+        <f t="shared" ref="J2:J62" si="2">(C2)/I2</f>
         <v>0</v>
       </c>
       <c r="K2" s="26">
-        <f t="shared" ref="K2:K60" si="3">(E2)/I2</f>
+        <f t="shared" ref="K2:K62" si="3">(E2)/I2</f>
         <v>0</v>
       </c>
       <c r="L2" s="17"/>
@@ -5996,11 +6020,11 @@
         <v>51</v>
       </c>
       <c r="Q45" s="35">
-        <f t="shared" ref="Q45:Q60" si="17">M45*C45</f>
+        <f t="shared" ref="Q45:Q62" si="17">M45*C45</f>
         <v>0</v>
       </c>
       <c r="R45" s="35">
-        <f t="shared" ref="R45:R60" si="18">M45*D45</f>
+        <f t="shared" ref="R45:R62" si="18">M45*D45</f>
         <v>0</v>
       </c>
       <c r="T45" s="7">
@@ -6079,7 +6103,7 @@
         <v>6</v>
       </c>
       <c r="O46" s="34">
-        <f t="shared" ref="O46:O60" si="21">M46+N46</f>
+        <f t="shared" ref="O46:O62" si="21">M46+N46</f>
         <v>25.5</v>
       </c>
       <c r="Q46" s="35">
@@ -7056,13 +7080,13 @@
         <v>32</v>
       </c>
       <c r="U57" s="38">
-        <f t="shared" ref="U57:U60" si="23">CEILING(MAX(0,90-MAX(K57,60))*I57/T57,1)*T57</f>
+        <f t="shared" ref="U57:U62" si="23">CEILING(MAX(0,90-MAX(K57,60))*I57/T57,1)*T57</f>
         <v>64</v>
       </c>
       <c r="V57" s="37"/>
       <c r="W57" s="37"/>
       <c r="X57" s="38">
-        <f t="shared" ref="X57:X60" si="24">MIN(CEILING(MAX(0,70-MAX(J57,30))*I57/T57,1)*T57,D57)</f>
+        <f t="shared" ref="X57:X62" si="24">MIN(CEILING(MAX(0,70-MAX(J57,30))*I57/T57,1)*T57,D57)</f>
         <v>0</v>
       </c>
       <c r="Y57" s="37"/>
@@ -7347,8 +7371,180 @@
         <v>45</v>
       </c>
     </row>
-    <row r="61" ht="25" customHeight="1"/>
-    <row r="62" ht="25" customHeight="1"/>
+    <row r="61" ht="25" customHeight="1" spans="1:34">
+      <c r="A61" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="C61" s="9">
+        <v>0</v>
+      </c>
+      <c r="D61" s="9">
+        <v>0</v>
+      </c>
+      <c r="E61" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F61" s="7">
+        <v>0</v>
+      </c>
+      <c r="G61" s="7">
+        <v>0</v>
+      </c>
+      <c r="H61" s="26">
+        <f>MAX(E61,F61)*1.375</f>
+        <v>0</v>
+      </c>
+      <c r="I61" s="26">
+        <v>1</v>
+      </c>
+      <c r="J61" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K61" s="26">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="M61" s="7">
+        <v>18</v>
+      </c>
+      <c r="N61" s="17">
+        <v>6</v>
+      </c>
+      <c r="O61" s="34">
+        <f t="shared" si="21"/>
+        <v>24</v>
+      </c>
+      <c r="Q61" s="35">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="R61" s="35">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="T61" s="7">
+        <v>20</v>
+      </c>
+      <c r="U61" s="38">
+        <f t="shared" si="23"/>
+        <v>40</v>
+      </c>
+      <c r="V61" s="37"/>
+      <c r="W61" s="37"/>
+      <c r="X61" s="38">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="Y61" s="37"/>
+      <c r="Z61" s="37"/>
+      <c r="AD61" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="AE61" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="AF61" s="7">
+        <v>25</v>
+      </c>
+      <c r="AG61" s="7">
+        <v>37</v>
+      </c>
+      <c r="AH61" s="7">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="62" ht="25" customHeight="1" spans="1:34">
+      <c r="A62" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="C62" s="9">
+        <v>0</v>
+      </c>
+      <c r="D62" s="9">
+        <v>0</v>
+      </c>
+      <c r="E62" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F62" s="7">
+        <v>0</v>
+      </c>
+      <c r="G62" s="7">
+        <v>0</v>
+      </c>
+      <c r="H62" s="26">
+        <f>MAX(E62,F62)*1.375</f>
+        <v>0</v>
+      </c>
+      <c r="I62" s="26">
+        <v>1</v>
+      </c>
+      <c r="J62" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K62" s="26">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="M62" s="7">
+        <v>18</v>
+      </c>
+      <c r="N62" s="17">
+        <v>6</v>
+      </c>
+      <c r="O62" s="34">
+        <f t="shared" si="21"/>
+        <v>24</v>
+      </c>
+      <c r="Q62" s="35">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="R62" s="35">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="T62" s="7">
+        <v>20</v>
+      </c>
+      <c r="U62" s="38">
+        <f t="shared" si="23"/>
+        <v>40</v>
+      </c>
+      <c r="V62" s="37"/>
+      <c r="W62" s="37"/>
+      <c r="X62" s="38">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="Y62" s="37"/>
+      <c r="Z62" s="37"/>
+      <c r="AD62" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="AE62" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="AF62" s="7">
+        <v>25</v>
+      </c>
+      <c r="AG62" s="7">
+        <v>37</v>
+      </c>
+      <c r="AH62" s="7">
+        <v>40</v>
+      </c>
+    </row>
     <row r="63" ht="25" customHeight="1"/>
     <row r="64" ht="25" customHeight="1"/>
     <row r="65" ht="25" customHeight="1"/>
@@ -7359,10 +7555,54 @@
     <row r="70" ht="25" customHeight="1"/>
     <row r="71" ht="25" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:AH54">
+  <autoFilter ref="A1:AH60">
     <extLst/>
   </autoFilter>
   <conditionalFormatting sqref="J45">
+    <cfRule type="cellIs" dxfId="0" priority="108" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="107" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="106" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K45">
+    <cfRule type="cellIs" dxfId="0" priority="105" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="104" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="103" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J46">
+    <cfRule type="cellIs" dxfId="0" priority="102" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="101" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="100" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K46">
+    <cfRule type="cellIs" dxfId="0" priority="99" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="98" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="97" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J47">
     <cfRule type="cellIs" dxfId="0" priority="96" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7373,7 +7613,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K45">
+  <conditionalFormatting sqref="K47">
     <cfRule type="cellIs" dxfId="0" priority="93" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7384,139 +7624,161 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J46">
+  <conditionalFormatting sqref="J48">
     <cfRule type="cellIs" dxfId="0" priority="90" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="89" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="1" priority="86" operator="lessThanOrEqual">
       <formula>60</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="88" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="2" priority="82" operator="greaterThanOrEqual">
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K46">
+  <conditionalFormatting sqref="K48">
+    <cfRule type="cellIs" dxfId="0" priority="78" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="74" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="70" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J49">
+    <cfRule type="cellIs" dxfId="0" priority="89" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="85" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="81" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K49">
+    <cfRule type="cellIs" dxfId="0" priority="77" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="73" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="69" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J50">
+    <cfRule type="cellIs" dxfId="0" priority="88" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="84" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="80" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K50">
+    <cfRule type="cellIs" dxfId="0" priority="76" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="72" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="68" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J51">
     <cfRule type="cellIs" dxfId="0" priority="87" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="86" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="85" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J47">
-    <cfRule type="cellIs" dxfId="0" priority="84" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="83" operator="lessThanOrEqual">
       <formula>60</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="82" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K47">
-    <cfRule type="cellIs" dxfId="0" priority="81" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="80" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="2" priority="79" operator="greaterThanOrEqual">
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J48">
-    <cfRule type="cellIs" dxfId="0" priority="78" operator="lessThanOrEqual">
+  <conditionalFormatting sqref="K51">
+    <cfRule type="cellIs" dxfId="0" priority="75" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="74" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="1" priority="71" operator="lessThanOrEqual">
       <formula>60</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="70" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="2" priority="67" operator="greaterThanOrEqual">
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K48">
+  <conditionalFormatting sqref="J52">
+    <cfRule type="cellIs" dxfId="0" priority="60" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="59" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="58" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K52">
+    <cfRule type="cellIs" dxfId="0" priority="57" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="56" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="55" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J53">
+    <cfRule type="cellIs" dxfId="0" priority="54" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="53" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="52" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K53">
+    <cfRule type="cellIs" dxfId="0" priority="51" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="50" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="49" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J54">
     <cfRule type="cellIs" dxfId="0" priority="66" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="65" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="64" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K54">
+    <cfRule type="cellIs" dxfId="0" priority="63" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="62" operator="lessThanOrEqual">
       <formula>60</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="58" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="2" priority="61" operator="greaterThanOrEqual">
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J49">
-    <cfRule type="cellIs" dxfId="0" priority="77" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="73" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="69" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K49">
-    <cfRule type="cellIs" dxfId="0" priority="65" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="61" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="57" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J50">
-    <cfRule type="cellIs" dxfId="0" priority="76" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="72" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="68" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K50">
-    <cfRule type="cellIs" dxfId="0" priority="64" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="60" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="56" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J51">
-    <cfRule type="cellIs" dxfId="0" priority="75" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="71" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="67" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K51">
-    <cfRule type="cellIs" dxfId="0" priority="63" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="59" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="55" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J52">
+  <conditionalFormatting sqref="J55">
     <cfRule type="cellIs" dxfId="0" priority="48" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7527,7 +7789,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K52">
+  <conditionalFormatting sqref="K55">
     <cfRule type="cellIs" dxfId="0" priority="45" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7538,7 +7800,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J53">
+  <conditionalFormatting sqref="J56">
     <cfRule type="cellIs" dxfId="0" priority="42" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7549,7 +7811,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K53">
+  <conditionalFormatting sqref="K56">
     <cfRule type="cellIs" dxfId="0" priority="39" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7560,29 +7822,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J54">
-    <cfRule type="cellIs" dxfId="0" priority="54" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="53" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="52" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K54">
-    <cfRule type="cellIs" dxfId="0" priority="51" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="50" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="49" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J55">
+  <conditionalFormatting sqref="J57">
     <cfRule type="cellIs" dxfId="0" priority="36" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7593,7 +7833,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K55">
+  <conditionalFormatting sqref="K57">
     <cfRule type="cellIs" dxfId="0" priority="33" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7604,7 +7844,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J56">
+  <conditionalFormatting sqref="J58">
     <cfRule type="cellIs" dxfId="0" priority="30" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7615,7 +7855,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K56">
+  <conditionalFormatting sqref="K58">
     <cfRule type="cellIs" dxfId="0" priority="27" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7626,7 +7866,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J57">
+  <conditionalFormatting sqref="J59">
     <cfRule type="cellIs" dxfId="0" priority="24" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7637,7 +7877,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K57">
+  <conditionalFormatting sqref="K59">
     <cfRule type="cellIs" dxfId="0" priority="21" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7648,7 +7888,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J58">
+  <conditionalFormatting sqref="J60">
     <cfRule type="cellIs" dxfId="0" priority="18" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7659,7 +7899,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K58">
+  <conditionalFormatting sqref="K60">
     <cfRule type="cellIs" dxfId="0" priority="15" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7670,7 +7910,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J59">
+  <conditionalFormatting sqref="J61">
     <cfRule type="cellIs" dxfId="0" priority="12" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7681,7 +7921,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K59">
+  <conditionalFormatting sqref="K61">
     <cfRule type="cellIs" dxfId="0" priority="9" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7692,7 +7932,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J60">
+  <conditionalFormatting sqref="J62">
     <cfRule type="cellIs" dxfId="0" priority="6" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7703,7 +7943,7 @@
       <formula>105</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K60">
+  <conditionalFormatting sqref="K62">
     <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
@@ -7715,6 +7955,39 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J29">
+    <cfRule type="cellIs" dxfId="2" priority="121" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="122" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="123" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J30:J44">
+    <cfRule type="cellIs" dxfId="2" priority="115" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="116" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="117" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:K29">
+    <cfRule type="cellIs" dxfId="2" priority="112" operator="greaterThanOrEqual">
+      <formula>105</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="113" operator="lessThanOrEqual">
+      <formula>60</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="114" operator="lessThanOrEqual">
+      <formula>70</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K30:K44">
     <cfRule type="cellIs" dxfId="2" priority="109" operator="greaterThanOrEqual">
       <formula>105</formula>
     </cfRule>
@@ -7722,39 +7995,6 @@
       <formula>60</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="0" priority="111" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J30:J44">
-    <cfRule type="cellIs" dxfId="2" priority="103" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="104" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="105" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K29">
-    <cfRule type="cellIs" dxfId="2" priority="100" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="101" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="102" operator="lessThanOrEqual">
-      <formula>70</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K30:K44">
-    <cfRule type="cellIs" dxfId="2" priority="97" operator="greaterThanOrEqual">
-      <formula>105</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="98" operator="lessThanOrEqual">
-      <formula>60</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="99" operator="lessThanOrEqual">
       <formula>70</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Restore dist assets and templates
</commit_message>
<xml_diff>
--- a/dist/产品库存及周转统计.xlsx
+++ b/dist/产品库存及周转统计.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="23040"/>
+    <workbookView windowHeight="15240"/>
   </bookViews>
   <sheets>
     <sheet name="产品库存" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">产品库存!$A$1:$AH$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">产品库存!$A$1:$AH$60</definedName>
   </definedNames>
   <calcPr calcId="144525" concurrentCalc="0"/>
 </workbook>
@@ -5941,11 +5941,11 @@
         <v>0</v>
       </c>
       <c r="T44" s="7">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="U44" s="38">
         <f t="shared" si="14"/>
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="V44" s="37"/>
       <c r="W44" s="37"/>
@@ -5962,7 +5962,7 @@
         <v>205</v>
       </c>
       <c r="AF44" s="7">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="AG44" s="7">
         <v>37</v>
@@ -7555,7 +7555,7 @@
     <row r="70" ht="25" customHeight="1"/>
     <row r="71" ht="25" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:AH62">
+  <autoFilter ref="A1:AH60">
     <extLst/>
   </autoFilter>
   <conditionalFormatting sqref="J45">

</xml_diff>

<commit_message>
Sync dist workbook from public
</commit_message>
<xml_diff>
--- a/dist/产品库存及周转统计.xlsx
+++ b/dist/产品库存及周转统计.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15240"/>
+    <workbookView windowHeight="23040"/>
   </bookViews>
   <sheets>
     <sheet name="产品库存" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">产品库存!$A$1:$AH$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">产品库存!$A$1:$AH$62</definedName>
   </definedNames>
   <calcPr calcId="144525" concurrentCalc="0"/>
 </workbook>
@@ -5941,11 +5941,11 @@
         <v>0</v>
       </c>
       <c r="T44" s="7">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="U44" s="38">
         <f t="shared" si="14"/>
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="V44" s="37"/>
       <c r="W44" s="37"/>
@@ -5962,7 +5962,7 @@
         <v>205</v>
       </c>
       <c r="AF44" s="7">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AG44" s="7">
         <v>37</v>
@@ -7555,7 +7555,7 @@
     <row r="70" ht="25" customHeight="1"/>
     <row r="71" ht="25" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:AH60">
+  <autoFilter ref="A1:AH62">
     <extLst/>
   </autoFilter>
   <conditionalFormatting sqref="J45">

</xml_diff>